<commit_message>
docs(owner): keep sample remits and practice contacts out of the repo [R-15.1]
AI-Assisted: true

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016DuG6tahaoPeUDXe9BDp4v
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -910,7 +910,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Share de-identified sample 835 remits and payer denial letters (or confirm synthetic only).</t>
+          <t>Decide whether real sample 835 remits/denial letters will ever be used (default: synthetic only); if yes, counsel-approved de-identification and an intake path first.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Sample files (no PHI) or confirmation.</t>
+          <t>Decision only. Never commit samples or attach them to this sheet.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Names/contacts of willing practices (no PHI).</t>
+          <t>Pointer to where contacts are kept outside the repo (e.g. CRM); no names here.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix(owner): dedupe dropdowns, validate inputs, reject unknown IDs, block formula injection [R-15]
AI-Assisted: true

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016DuG6tahaoPeUDXe9BDp4v
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -1591,16 +1591,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:L21"/>
-  <dataValidations count="6">
-    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"P0,P1,P2,P3"</formula1>
-    </dataValidation>
-    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Data source,Clarification,Decision,Legal/Compliance,Vendor/Account,Design/Brand,Business"</formula1>
-    </dataValidation>
+  <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
docs(appeals): tick A1 checkboxes, update roadmap and owner items [R-4.2.1]
Ticks the appeals.md A1 acceptance criteria, marks the appeals lines done in
ROADMAP.md, adds a PROJECT_STATE entry, and records five owner decisions from
the spec's open questions (late-filing blocking, withdrawn/dismissed denial
mapping, appeal version history, Medicare amount-in-controversy source, and
field masking) as OA-021..OA-025 in OWNER_ACTION_ITEMS.xlsx.

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fj8yp8DTKLRN898BysVFAr
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1589,8 +1589,278 @@
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr"/>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>OA-021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Confirm whether a late appeal submission (past the computed deadline) should be blocked, warned, or only recorded and flagged.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>A1 records and flags; a human should confirm this before A2/A3 lock in stricter behavior.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Decision: block / warn / record-and-flag (current default).</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>specs/appeals.md</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>appeals A1 agent</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Before A2</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>OA-022</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Confirm the withdrawn/dismissed decision outcome's mapping to a denial status (A1 default: both set the denial to 'closed' with a required reason).</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>A withdrawal for a procedural reason may need to stay distinguishable from a dismissal on the merits.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Decision to keep the A1 default or add a distinct denial status/flag.</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>specs/appeals.md</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>appeals A1 agent</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Before A2/A3</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>OA-023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Decide if an appeal needs its own immutable version history (like claim_versions) once A2 adds an editable letter body.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Shapes whether A2 needs a new history table before shipping editable letter content.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Yes/no decision.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>specs/appeals.md</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>appeals A1 agent</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Before A2</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>OA-024</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Provide a source and an annual-update owner for Medicare appeal amount-in-controversy thresholds (REQUIREMENTS §4.2, QIC/ALJ/Council/federal court).</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>rules/catalog.ts cannot encode the higher Medicare appeal levels' thresholds without a cited source.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Citation/source + who keeps it current.</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>specs/appeals.md; rules/</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>appeals A1 agent</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Before A3</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>OA-025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Clarification</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Confirm whether any role/field visibility rule beyond the existing claim/denial matrix should mask an appeal's tracking_reference or recovered_cents.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Confirms R-5.1.2 coverage extends correctly to the new appeal fields.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Yes/no per field, or 'no change'.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>specs/appeals.md; R-5.1.2</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>appeals A1 agent</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Before A2</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L21"/>
+  <autoFilter ref="A1:L26"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
feat(remittances): reversals and denial capture from posted 835s [R-3.10.3, §8.3]
Reversals (CLP02 22) load and post: paid total drops with a claim version,
and the reversed payment is marked recorded in error on the prompt-pay
clock. Posting captures one denial per unexpected adjustment (not PR or
CO-45), linked to its remittance, with the appeal deadline from the rules
engine. Server-side balance check on post; the database refuses spoofed
remittance history rows. Owner items OA-021 (CARC mapping) and OA-022
(interest accrual).

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XZZBf2BeNYZZSKvbQRh75J
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1589,8 +1589,116 @@
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr"/>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>OA-021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Clarification</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Confirm (or have a biller/counsel confirm) how each CARC maps to a denial category, and which adjustments count as denials versus expected reductions (DenialDesk treats PR and CO-45 as expected).</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Remittance posting now captures denials automatically; the category drives the work queue and appeal routing.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Reviewed CARC → category table (src/domain/carc.ts) and the expected-adjustment list, with source.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>R-3.10.1, specs/remittances-and-prompt-pay.md (R2)</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>agent R2 2026-09-26</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Before real remittances</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>OA-022</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Clarification</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Confirm how late-payment interest should start (payment due date) and whether it accrues on claims still unpaid.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Prompt-pay interest worksheet and totals depend on it (currently pending counsel verification).</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Counsel answer with citation (§ 627.6131 interest subsection).</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>R-3.1.3, rules/prompt-pay.ts</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>agent R2 2026-09-26</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Before production</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L21"/>
+  <autoFilter ref="A1:L23"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
docs(appeals): document practice_settings, record owner items from review [R-4.2.1]
Documents the practice_settings table and appeal_notes' insert/select-only
RLS in appeals.md, notes the new composite FK/trigger on the appeals table,
and records five owner decisions from the A1 review round (OA-026..OA-030):
abandoning a draft appeal, compliance member-ID reveal, counsel sign-off on
the level 2-5 Medicare rules, sensitivity-tag masking timing, and appeal
record retention.

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fj8yp8DTKLRN898BysVFAr
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1859,8 +1859,278 @@
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
     </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>OA-026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Clarification</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Confirm whether a draft (or in_review/ready) appeal that's never submitted can be abandoned/withdrawn, or must always move to submitted before it can be closed out.</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>The A1 status trigger only allows withdrawn/dismissed from submitted or awaiting_decision; an abandoned draft currently has no exit path.</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Decision: add a draft-cancel transition, or confirm drafts must always be submitted or left open.</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>specs/appeals.md</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>appeals A1 review</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Before A2</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>OA-027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Confirm compliance's read-only role on appeals still permits full member-ID reveal, consistent with (or overriding) the same open question on denials/claims (R-5.1.2).</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Appeals reuse the denial/claim role matrix; an unresolved compliance-visibility decision there also applies here.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Decision: compliance sees masked-only, or full reveal like other roles.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>specs/appeals.md; R-5.1.2</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>appeals A1 review</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Before real data</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>OA-028</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Legal/Compliance</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Counsel sign-off on the Medicare appeal-level rules added for levels 2-5: the 5-day receipt presumption applied to QIC/ALJ/Council/federal court (not yet confirmed for those levels the way it is for redetermination), the federal-court citation (42 CFR 405.1132 vs 405.1136(c)), and the amount-in-controversy thresholds (42 CFR 405.1006, currently unsourced).</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>All of rules/catalog.ts's levels 2-5 rules are flagged VERIFY; A3 cannot compute a level 2-5 deadline for real practices without this.</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed citations/values, or corrections, per rule ID.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>rules/catalog.ts; rules/deadlines.ts</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>appeals A1 review</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Before A3</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>OA-029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Decide whether sensitivity-tag masking (HIV, SUD/Part 2, etc.) should be enforced on the appeal and denial detail pages now, or deferred with the rest of the sensitivity-tag work (R-3.5.1).</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Appeals show the same patient/claim fields as denials, which don't yet enforce sensitivity tags.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Decision: enforce now (adds scope to A2) or defer (tracked with the existing sensitivity-tag gap).</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>specs/appeals.md; R-3.5.1</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>appeals A1 review</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Before real data</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>OA-030</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Confirm the retention period for appeal records (appeals, appeal_notes) once a real retention policy exists.</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>No retention/legal-hold policy is defined yet for the new tables, same gap as claims/denials.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Retention period or pointer to the practice's policy.</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>specs/appeals.md</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>appeals A1 review</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Before real data</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L26"/>
+  <autoFilter ref="A1:L31"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
docs(rules): P1 acceptance criteria, owner answers, counsel item OA-023 [R-15.6]
AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014AdmDiNviiZEgKywuEWuUg
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1697,8 +1697,62 @@
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
     </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>OA-023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Legal/Compliance</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Have Florida healthcare counsel confirm the deadline-computation readings now encoded in rules/: (1) whether Fla. R. Gen. Prac. &amp; Jud. Admin. 2.514 weekend/holiday roll-forward applies to prompt-pay and timely-filing clocks outside court, and which Florida holiday list governs (§ 110.117 vs § 683.01); (2) the meaning of 'month' under Fla. Stat. § 1.01 and end-of-month clamping (Aug 31 + 6 months = Feb 28/29); (3) date of service vs date of discharge as the timely-filing anchor for inpatient claims; (4) that Medicare Advantage is outside Florida prompt pay (plan contract; 42 CFR 422.520 30-day clean-claim rule for non-contracted providers); (5) interest starting the first calendar day after the prompt-pay deadline; (6) Medicare 1-year filing with next-federal-workday roll-forward.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Every computed deadline on the claims, denials and prompt-pay pages depends on these readings; all stay VERIFY until confirmed.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Counsel answer per item with citation; then a human records confirmedBy on each rule.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>R-15.6, R-3.1.1, R-3.1.3, R-3.1.5, R-4.2.1, specs/rules-engine-skeleton.md</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>florida-rules-engine 2026-09-26</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Before production</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L23"/>
+  <autoFilter ref="A1:L24"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
docs(rules): record option-1 roll-forward decision, OA-023 item 7, D2 follow-up [R-15.6]
AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014AdmDiNviiZEgKywuEWuUg
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -1720,7 +1720,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Have Florida healthcare counsel confirm the deadline-computation readings now encoded in rules/: (1) whether Fla. R. Gen. Prac. &amp; Jud. Admin. 2.514 weekend/holiday roll-forward applies to prompt-pay and timely-filing clocks outside court, and which Florida holiday list governs (§ 110.117 vs § 683.01); (2) the meaning of 'month' under Fla. Stat. § 1.01 and end-of-month clamping (Aug 31 + 6 months = Feb 28/29); (3) date of service vs date of discharge as the timely-filing anchor for inpatient claims; (4) that Medicare Advantage is outside Florida prompt pay (plan contract; 42 CFR 422.520 30-day clean-claim rule for non-contracted providers); (5) interest starting the first calendar day after the prompt-pay deadline; (6) Medicare 1-year filing with next-federal-workday roll-forward.</t>
+          <t>Have Florida healthcare counsel confirm the deadline-computation readings now encoded in rules/: (1) whether Fla. R. Gen. Prac. &amp; Jud. Admin. 2.514 weekend/holiday roll-forward applies to prompt-pay and timely-filing clocks outside court, and which Florida holiday list governs (§ 110.117 vs § 683.01); (2) the meaning of 'month' under Fla. Stat. § 1.01 and end-of-month clamping (Aug 31 + 6 months = Feb 28/29); (3) date of service vs date of discharge as the timely-filing anchor for inpatient claims; (4) that Medicare Advantage is outside Florida prompt pay (plan contract; 42 CFR 422.520 30-day clean-claim rule for non-contracted providers); (5) interest starting the first calendar day after the prompt-pay deadline; (6) Medicare 1-year filing with next-federal-workday roll-forward. (7) accept or reject the engineering choice (not an owner decision) to apply the reading attributes anchor, rollForward, side and confirmedBy, and the FL insurer/HMO split, to the baseline rule versions instead of adding new effective-dated versions. Until (1) is confirmed, the owner chose option 1 (2026-09-27): the unrolled date governs for provider-side and payer-side deadlines; the rolled date is shown as 'pending counsel' only. After confirmation a human adds a confirmed version to ROLL_FORWARD_POLICY in rules/roll-forward.ts.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1748,7 +1748,11 @@
           <t>Before production</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27: option 1 chosen (conservative/unrolled date governs until counsel confirms roll-forward).</t>
+        </is>
+      </c>
       <c r="L24" s="2" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(university): DenialDesk University courses with per-user completion record [R-10.4]
In-app training reachable from a "University" link in the global header and a
"DenialDesk University" item in the user menu (owner request). Five courses
authored as typed lesson blocks in src/domain/university/catalog.ts; every legal
value is a `rules` block resolved from rules/catalog.ts at render time with its
citation and verification badge (a unit test rejects statutory numbers typed in
prose), and CARC meanings come from src/domain/carc.ts. Per-user completions in
`university_progress` (migration 0033; RLS, app role SELECT/INSERT only, member
FK) are audited as `university.lesson_completed`. Spec, roadmap, design guide,
project state, and owner action item OA-034 updated.

AI-Assisted: true
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CuA9GJV653ZDZe8uQunkQh
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2291,8 +2291,62 @@
       <c r="K34" s="2" t="inlineStr"/>
       <c r="L34" s="2" t="inlineStr"/>
     </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>OA-034</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Clarification</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Decide whether DenialDesk University lesson completions should serve as HIPAA training evidence for practices, and in what form (per-user table under Settings, .xlsx export).</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Sets the scope of University U3 (practice training record) and whether it counts toward R-10.4.</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Yes/no, the practice roles who may see it, and any required fields (e.g. annual re-take).</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>R-10.4; specs/denialdesk-university.md U3</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>university session 2026-09-27</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Before U3</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr"/>
+      <c r="L35" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L34"/>
+  <autoFilter ref="A1:L35"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
fix(i18n): review follow-ups: English CSV headers in import errors, translated CSV/835 diagnostics, date-only columns, tests [R-11.1]
Import errors quote the English CSV header contract; CsvError carries a
code the importers translate; 835 parser diagnostics sit inside a
translated sentence; voucher month names and the root metadata follow the
language; five Created columns are date-only again; Portuguese zero counts
read plural; timeout minutes come from policy; compliance wording fixes
(citations, VERIFY token, BAA and signer labels, money format). Tests for
getLocale, setLocale, rich(), Spanish import errors and sheets, and the
users.locale CHECK constraint.

AI-Assisted: true

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JwjCviBKhorAsLxiey3BFh
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="214">
   <si>
     <t>ID</t>
   </si>
@@ -649,13 +649,16 @@
     <t>Review</t>
   </si>
   <si>
-    <t>Native-speaker review of the Spanish and Portuguese billing terminology used across the product (glossary in specs/internationalization.md).</t>
+    <t>Native-speaker review of the Spanish and Portuguese billing terminology (glossary in specs/internationalization.md), plus counsel/compliance sign-off that translated attestations and caveats (synthetic-data attestation, BAA recording labels, uncontestable-obligation alert, R-8.7 suppression and residual-risk text) mean the same thing in law.</t>
   </si>
   <si>
     <t>The agent-authored translations use U.S. Spanish and Brazilian Portuguese billing vocabulary (reclamación / reivindicação, denegación / negativa, apelación / recurso, remesa / remessa). A biller who works in those languages should confirm the terms match what Florida practices actually say before launch.</t>
   </si>
   <si>
     <t>Confirmed or corrected glossary rows; any screen wording to change.</t>
+  </si>
+  <si>
+    <t>Before the Azure (production) launch</t>
   </si>
 </sst>
 </file>
@@ -2230,7 +2233,7 @@
         <v>13</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>87</v>
+        <v>43</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>209</v>
@@ -2251,7 +2254,7 @@
         <v>206</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>74</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(university): University of DenialDesk logo button in the header and on the welcome page [R-10.4, §11]
Mirrors the Wiki wordmark button: the owner's "University of DenialDesk" logo,
white background removed and otherwise unaltered, replaces the graduation-cap
text link in the global header and the welcome page's text link. Accessible
name "University of DenialDesk"; aria-current logic unchanged. The header's
practice block now shows from 1280px (it stays in the user menu below that) so
both logo buttons fit a 1024px window with a long user name. Brand README,
specs (university, welcome page, ERP shell), DESIGN.md, e2e selectors, and
OA-037 (license / tool, now covering both logos) updated.

AI-Assisted: true
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CuA9GJV653ZDZe8uQunkQh
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -2480,7 +2480,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Confirm the license and generating tool for the DenialDesk Wiki wordmark (public/brand/denialdesk-wiki.png) and that DenialDesk holds the rights to use the logo mark in it.</t>
+          <t>Confirm the license and generating tool for the DenialDesk Wiki wordmark (public/brand/denialdesk-wiki.png) and the University of DenialDesk logo (public/brand/university-of-denialdesk.png), and that DenialDesk holds the rights to use the logo mark in them.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2490,7 +2490,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>License/rights confirmation and the tool used, noted in public/brand/README.md.</t>
+          <t>License/rights confirmation and the tool used for each, noted in public/brand/README.md.</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix(university): review fixes for the logo button; counsel item on the "University" name [R-10.4, §11]
The Wiki's welcome article and the Wiki, project-state docs no longer describe
the removed "University" text link. The 1024px shell test now asserts both logo
buttons are visible and the practice block appears only from 1280px. OA-037
covers both logos; OA-038 asks counsel whether "University" may be used in the
name under Florida law.

AI-Assisted: true
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CuA9GJV653ZDZe8uQunkQh
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2485,7 +2485,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>The wordmark is shown in the header on every signed-in screen; its provenance is unrecorded (same open question as the reception image).</t>
+          <t>Both logos are shown in the header on every signed-in screen and on the welcome page; their provenance is unrecorded (same open question as the reception image).</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -2495,7 +2495,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>docs/specs/university-wiki.md, DESIGN.md §4</t>
+          <t>docs/specs/university-wiki.md, docs/specs/denialdesk-university.md, DESIGN.md §4, public/brand/README.md</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2511,8 +2511,62 @@
       <c r="K38" s="2" t="inlineStr"/>
       <c r="L38" s="2" t="inlineStr"/>
     </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>OA-038</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Legal/Compliance</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Ask counsel whether calling the training center "University of DenialDesk" / "DenialDesk University" is permitted under Florida rules on the use of "university" in a name (Fla. Stat. ch. 1005, Commission for Independent Education) or needs a different name before launch.</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>The name appears in the app header, welcome page, and user menu; renaming later would touch the logo, copy, and URLs.</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Counsel's answer; if a rename is needed, the new name.</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>specs/denialdesk-university.md; public/brand/README.md</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>compliance-checker 2026-09-27</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Before launch</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L38"/>
+  <autoFilter ref="A1:L39"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
feat(home): revamp the home page with live totals and a step pipeline [§11, R-11.1]
- Header band gains a live strip of practice denial totals (open, amount at
  risk, due soon, past deadline) from queueSummary, each cell linking to the
  Overview or queue. Aggregates only: no rows, no PHI, no audit event (OA-044
  asks the owner to confirm).
- The two step flows become a connected pipeline (FlowSteps): module tile per
  step, solid connector between shipped steps, dashed next to planned ones,
  whole shipped cell clickable, "N of M steps available".
- "Your modules" becomes a card grid with page counts and page links;
  safeguard icons sit on teal tiles.
- Hover feedback only (150ms, off under reduced motion); new strings in
  English, Spanish, and Portuguese; E2E covers the strip and counts.

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E2eUayMWvXD783hH72B9Zi
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$44</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2786,8 +2786,62 @@
       <c r="K43" s="3" t="inlineStr"/>
       <c r="L43" s="3" t="inlineStr"/>
     </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>OA-044</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Legal/Compliance</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Confirm that practice-wide denial totals without identifiers (counts and sums on the home page) are not a PHI read and need no audit event.</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>The home page revamp shows live open-denial totals without auditing each view; Insight reports audit aggregates as PHI-adjacent, so the rule should be set once.</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>Yes/no; if no, the agent adds an audit event to the home page strip.</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>R-7.5.1; specs/welcome-page.md</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>home-page revamp session 2026-09-27</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>Before the Azure (production) launch</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr"/>
+      <c r="L44" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L43"/>
+  <autoFilter ref="A1:L44"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
docs(owner): add OA-057 cross-practice EHR connection safeguard [R-7.2.4]
AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NY7r13quPdzAWKCKUiLCt2
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$57</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3488,8 +3488,62 @@
       <c r="K56" s="3" t="inlineStr"/>
       <c r="L56" s="3" t="inlineStr"/>
     </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>OA-057</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Confirm the safeguard against one practice pulling another practice's EHR patients: the platform operator approves every real EHR connection after checking its address and client ID with the practice's EHR administrator, the same EHR registration can't be used by two practices, and each connection gets its own signing key where the EHR vendor supports it.</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>Security review 2026-09-28 (Critical C1): with one shared DenialDesk signing key, a practice admin could enter another practice's EHR address and client ID and sync its patients.</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>Accept the three safeguards, or choose differently (e.g. per-practice keys only).</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>docs/specs/patient-integrations.md (OA-057); R-7.2.4</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>patient-integrations session 2026-09-28</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>Before PI1b</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr"/>
+      <c r="L57" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L56"/>
+  <autoFilter ref="A1:L57"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
docs(records): note unsubmitted-only name reads; log OA-060 [R-7.1.3, R-7.5.1]
Security-review Low: the unsubmitted index comments now say names are read only for the
unsubmitted group's patientName sort. Compliance-checker question (sort-only name reads vs. the
claim.list_viewed audit) logged for the owner as OA-060 and linked from PROJECT_STATE.

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HqLbpzoXVNQQkdAf7fz5qe
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$60</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3650,8 +3650,62 @@
       <c r="K59" s="3" t="inlineStr"/>
       <c r="L59" s="3" t="inlineStr"/>
     </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>OA-060</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Legal/Compliance</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>Confirm that patient names read only to order the unsubmitted claims queue by patient (never shown or returned beyond the displayed page) are covered by the claim.list_viewed audit event and need no separate audit event.</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>Settles whether sort-only PHI reads need their own audit trail (R-7.5.1) or only minimum-necessary handling (R-5.1.2).</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>Yes (covered) / No (add an audit event for sort-only reads).</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>R-7.5.1, R-5.1.2; specs/record-pages.md P4</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>compliance-checker 2026-09-28</t>
+        </is>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>Before launch</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr"/>
+      <c r="L60" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L59"/>
+  <autoFilter ref="A1:L60"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
docs(integrations): PI2a part 2 spec ticks, OA-062 (TLS 1.3 minimum), project state [R-7.3.1, R-7.3.4]
AI-Assisted: true

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01NY7r13quPdzAWKCKUiLCt2
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$62</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3758,8 +3758,62 @@
       <c r="K61" s="3" t="inlineStr"/>
       <c r="L61" s="3" t="inlineStr"/>
     </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>OA-062</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>Decide whether the FHIR transport should require TLS 1.3 as a minimum.</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>R-7.3.1 requires TLS 1.2+ and prefers 1.3. The transport allows 1.2 (ECDHE + AEAD suites only) and negotiates 1.3 when offered. Requiring 1.3 is stronger but would lock out EHR vendors that only support 1.2.</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>Keep TLS 1.2 minimum (current), or require 1.3 (and, if so, which vendors are known to be 1.2-only).</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>docs/specs/patient-integrations.md PI2a; R-7.3.1</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>agent 2026-09-28</t>
+        </is>
+      </c>
+      <c r="J62" s="3" t="inlineStr">
+        <is>
+          <t>Before the first real practice</t>
+        </is>
+      </c>
+      <c r="K62" s="3" t="inlineStr"/>
+      <c r="L62" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L61"/>
+  <autoFilter ref="A1:L62"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
docs(integrations): PI2a part 2 spec ticks, OA-063 (pre-production signing key), audit-log test record [R-7.3.4, R-7.3.5]
AI-Assisted: true

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01NY7r13quPdzAWKCKUiLCt2
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$63</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3812,8 +3812,62 @@
       <c r="K62" s="3" t="inlineStr"/>
       <c r="L62" s="3" t="inlineStr"/>
     </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>OA-063</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Vendor/Account</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>Generate a pre-production ES384 signing key and set it as INTEGRATION_SIGNING_KEY, a functions-only secret, in the Netlify site settings.</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>Test connection and the token request sign with this shared key, and its public half is published at /.well-known/jwks.json for a vendor sandbox administrator to register. Without it, Test connection reports that the signing key isn't configured. Never use it in production (production refuses it) and never commit it.</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>Confirmation that the secret is set for the Netlify functions only (not the build or the client), and the JWKS URL once it serves a key. Generate with: openssl ecparam -name secp384r1 -genkey -noout | openssl pkcs8 -topk8 -nocrypt (PKCS#8 PEM).</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>docs/specs/patient-integrations.md PI2a Keys; R-7.3.4, R-7.3.5</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>agent 2026-09-28</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>Before testing against a vendor sandbox</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr"/>
+      <c r="L63" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L62"/>
+  <autoFilter ref="A1:L63"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
docs(integrations): PR #87 compliance re-review notes; OA-065 for the Submit gate and shared pre-production key [R-7.3.4, R-7.3.5]
'Owner decision' wording becomes 'coordinator decision pending owner
confirmation (OA-065)'; Resume-from-error gate listed as still open; the
env-key event's sources described accurately; gate summary names the
token endpoint key; owner workbook auto-filter covers the new rows.

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NY7r13quPdzAWKCKUiLCt2
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$65</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3920,8 +3920,62 @@
       <c r="K64" s="2" t="n"/>
       <c r="L64" s="2" t="n"/>
     </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>OA-065</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Confirm two PI2a coordinator decisions: (a) Submit's Test-connection gate is stricter than the spec's plain wording — the newest test for the connection must be a pass within 24 h, bound to the tested base URL, client ID, token endpoint and key, issuer, and signing kid (a later failed test or transport refusal voids it); (b) pre-production signs every connection with one shared key (INTEGRATION_SIGNING_KEY), accepted as a pre-production exception with the operator verifying client_id ownership outside the app at approval.</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>(a) decides when a practice may submit a connection; (b) is a residual risk recorded in the threat model (S3): an admin who knows another practice's client_id at the same EHR could get a passing test for it. Synthetic data only; per-connection Key Vault keys remove it in production.</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Confirm (a) and (b) as built, or say what to change (e.g. 'any pass in 24 h counts').</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>docs/specs/patient-integrations.md (PI2a Test connection, Keys; PI1c Approve); docs/threat-models/patient-integrations.md S3; R-7.3.4, R-7.3.5</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>Coordinator (PR #87 compliance review), 2026-09-28</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>Before Submit ships (next PI2a PR)</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="n"/>
+      <c r="L65" s="2" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L62"/>
+  <autoFilter ref="A1:L65"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
ci(telemetry): image build reads .npmrc; owner row for the next dev update check [R-7.4.2, R-15.7]
Compliance re-review of PR #96:
- The Dockerfile deps stage copies .npmrc, so `pnpm install` in the
  image also skips the update check (docker build does not look like CI
  to pnpm); telemetry.test.ts checks it.
- The SC-A2.6 gap row now says what accepting the residual takes: a
  written, time-boxed exception ADR signed by the Security and Privacy
  Officers (HC §0). New owner row OA-079 asks for that decision (OA-078
  is claimed by PR #97).

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QCaBhuvNddsqynubD6Mpxq
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$75</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L74"/>
+  <dimension ref="A1:L75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4460,8 +4460,62 @@
       <c r="K74" s="2" t="n"/>
       <c r="L74" s="2" t="n"/>
     </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>OA-079</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>Legal/Compliance</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>Decide whether local development may keep Next.js's unavoidable 'next dev' update check (it asks registry.npmjs.org for newer Next.js versions; no opt-out in 16.3.6) under a written, time-boxed exception ADR signed by the Security and Privacy Officers (HC §0), or keep SC-A2.6 tracked as a known gap.</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>SC-A2.6 bans update checks; everything else that phones home is now off. No PHI is involved (local development holds synthetic data only).</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>Accept (officers sign an exception ADR the agent drafts) or keep tracked.</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>SC-A2.6; HC §0; PR #96</t>
+        </is>
+      </c>
+      <c r="I75" s="3" t="inlineStr">
+        <is>
+          <t>SC gap PRs session 2026-09-29</t>
+        </is>
+      </c>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>Before the first real practice</t>
+        </is>
+      </c>
+      <c r="K75" s="3" t="inlineStr"/>
+      <c r="L75" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L73"/>
+  <autoFilter ref="A1:L75"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
docs(integrations): ADR 0012, spec ticks, threat model, runbook, owner actions for background jobs [R-7.3.5, R-15.9]
ADR 0012 (Proposed) records background execution. The spec ticks PI2b Jobs, PI3
scheduled enqueue and the three-failure rule with Built notes (SIEM alerts stay
deferred). The threat model gains S5 detail, the job secret (S7), the jobs role and
functions (S8) and job floods (D5). PROJECT_STATE lists every privilege statement in
0044 for the R-15.9 sign-off. The Netlify runbook and .env.example document
INTEGRATION_JOB_SECRET. Owner actions OA-083 (sign-off) and OA-084 (secret, site
password check).

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NY7r13quPdzAWKCKUiLCt2
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$84</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -4894,8 +4894,116 @@
       <c r="K82" s="2" t="n"/>
       <c r="L82" s="2" t="n"/>
     </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>OA-083</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Legal/Compliance</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>Sign off (R-15.9) on migration 0044 before it runs anywhere beyond a local or test database: it creates the NOLOGIN role `denialdesk_jobs`, two SECURITY DEFINER functions (`integration_claim_run(uuid)`, `integration_enqueue_due_runs()`), and their GRANT and REVOKE statements. Every statement is listed verbatim in the PR description, docs/PROJECT_STATE.md and ADR 0012.</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>Background sync jobs need a database role that can do exactly two things: ask whether a run is a queued run of an active connection (and whose), and queue the 15-minute scheduled runs. The role has no table privilege, `denialdesk_app` is not granted either function, and PUBLIC is revoked first. The functions run as their owner and walk the practices one at a time under each practice's own row-level security policy (no policy or BYPASSRLS is added). The same migration also checks that the integration service-principal row seeded by 0043 is still disabled, has the non-hash password marker and no membership (security review L3), and stops the migration if not. Netlify has already applied 0001 to 0043; 0044 is new and pending.</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>Approve, or ask for a different shape (for example the claim as a plain function without the tenant walk, which needs a BYPASSRLS or superuser owner). Recorded on the PR.</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>docs/specs/patient-integrations.md (PI2b Jobs, PI3); docs/decisions/0012-background-execution.md; drizzle/0044_patient_integrations_jobs.sql; R-15.9</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>PI2c jobs builder, 2026-09-29</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>Before 0044 is merged (Netlify applies migrations on the next deploy)</t>
+        </is>
+      </c>
+      <c r="K83" s="2" t="n"/>
+      <c r="L83" s="2" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>OA-084</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Vendor/Account</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>Generate INTEGRATION_JOB_SECRET (at least 32 random bytes, for example `openssl rand -base64 48`) and set it as a functions-only secret in the Netlify site settings, then check that the site's own password protection does not block the function URL the app posts jobs to.</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>The secret signs every background sync job (HMAC-SHA256 over the body and a timestamp) and lets the worker refuse forged or replayed ones. Until it is set nothing breaks: Sync now keeps running in the request as before, and the worker and the 15-minute scheduled function refuse to run. Once it is set, Sync now queues a job by posting to this deploy's own `/.netlify/functions/integration-sync-background`, and the site is behind Netlify password protection. If that protection also covers function URLs the post is refused (a 401 from Netlify) and Sync now reports that the sync could not be started; the fix would then be an exemption for that path or a basic-auth header, which is a small follow-up. Scheduled functions run only on the published (production) deploy, not on deploy previews. Never commit the value; production keeps it in Key Vault.</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>Confirmation the secret is set for functions only (not the build or the client) and never pasted anywhere else; then, after the next deploy, press Sync now on the pre-production sandbox connection and confirm it says the sync was queued and a run appears in Sync history, and that a scheduled run appears within 15 minutes. Tell the agent if the press says it could not be started.</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>docs/specs/patient-integrations.md PI2b Jobs, PI3; docs/decisions/0012-background-execution.md; docs/runbooks/netlify.md; R-7.3.5</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>PI2c jobs builder, 2026-09-29</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>Before the first background sync on Netlify</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="n"/>
+      <c r="L84" s="2" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L82"/>
+  <autoFilter ref="A1:L84"/>
   <dataValidations count="6">
     <dataValidation sqref="B10:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
fix(claims): C2 last review items: contiguity marker, audit-failure safety, rate-limit test [§8.2, R-7.5.1]
- Only a valid claim number moves the contiguity marker, so A / invalid / A no
  longer reports claim_rows_not_contiguous (unit tests for invalid and blank).
- A failing audit write for reason "error" no longer replaces the original error.
- The rate-limit integration test fixes the clock mid-window (Date only) so a
  ten-minute boundary can't fall between the hits and the action.
- A test that never ran the import is renamed and reduced to a parser check.
- In-file matching pushes onto the bucket instead of copying it.
- Spec Tests box ticked (CI green on f3b233a); OA-084 gains the repeated-line and
  contiguity questions and notes that the rate limit counts refused attempts.

No migration, no GRANT, no new dependency.

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NY7r13quPdzAWKCKUiLCt2
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -4977,7 +4977,7 @@
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>Answer the C2 charge-import questions: (1) who counts as a biller (C2 uses admin, manager, specialist); (2) is a same-patient, same-payer, same-day, same-code-and-modifiers row always a duplicate, or does the practice need an override for a legitimate repeat service; (3) is one claim per Claim number right, or must one PM encounter split into several claims per payer; (4) which practice-management system exports will supply the file, so the columns can be mapped.</t>
+          <t>Answer the C2 charge-import questions: (1) who counts as a biller (C2 uses admin, manager, specialist); (2) is a same-patient, same-payer, same-day, same-code-and-modifiers row always a duplicate, or does the practice need an override for a legitimate repeat service; (3) is one claim per Claim number right, or must one PM encounter split into several claims per payer; (4) which practice-management system exports will supply the file, so the columns can be mapped; (5) can one claim legitimately carry the same line twice (for example the same J-code with different NDCs, or separate-line billing of the same service)? The import refuses a repeated procedure code plus modifiers on one claim, and there is no override yet; (6) is it acceptable that a claim's rows must be next to each other in the file (a claim number that comes back after other claims is refused), or do your PM exports interleave claims? Note: the import rate limit (10 per practice per 10 minutes) counts every attempt, refused ones included.</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
@@ -4987,7 +4987,7 @@
       </c>
       <c r="G84" s="3" t="inlineStr">
         <is>
-          <t>Answers to the four questions.</t>
+          <t>Answers to the four questions; answers to (5) and (6), and whether 10 attempts per 10 minutes is enough for a billing day.</t>
         </is>
       </c>
       <c r="H84" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(claims): C2 charge capture via CSV import → draft claims [§8.2, R-3.10.1, R-3.10.3, R-7.5.1] (#99)
Charge CSV upload at /claims/import creates draft claims through createDraftClaims
(version 1 + claim.created audit). All-or-nothing; codes stored exactly as given;
patients matched by MRN and never written; duplicate lines, claims and files refused;
timely filing warns only; per-practice lock and rate limit; synthetic-only guard.

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NY7r13quPdzAWKCKUiLCt2
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$84</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -59,12 +59,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -432,13 +435,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="7"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
@@ -4894,23 +4900,122 @@
       <c r="K82" s="2" t="n"/>
       <c r="L82" s="2" t="n"/>
     </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>OA-083</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>Decide whether a claim_imports table (file SHA-256, counts, importer, time) should be added so a re-uploaded charge file is caught by file identity; it needs a new table and a GRANT to denialdesk_app, so it needs your sign-off (R-15.9).</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>C2 charge import detects re-uploads by claim number only, so a file whose claim numbers were all changed is not recognised as the same file.</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>Approve or decline the table and its grant; if approved, the retention period for import history.</t>
+        </is>
+      </c>
+      <c r="H83" s="3" t="inlineStr">
+        <is>
+          <t>specs/claims.md C2</t>
+        </is>
+      </c>
+      <c r="I83" s="3" t="inlineStr">
+        <is>
+          <t>agent Claude C2 (vigilant-tesla-ps41e9), 2026-09-29</t>
+        </is>
+      </c>
+      <c r="J83" s="3" t="inlineStr">
+        <is>
+          <t>Before the first real practice</t>
+        </is>
+      </c>
+      <c r="K83" s="3" t="inlineStr"/>
+      <c r="L83" s="3" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>OA-084</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>Clarification</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>Answer the C2 charge-import questions: (1) who counts as a biller (C2 uses admin, manager, specialist); (2) is a same-patient, same-payer, same-day, same-code-and-modifiers row always a duplicate, or does the practice need an override for a legitimate repeat service; (3) is one claim per Claim number right, or must one PM encounter split into several claims per payer; (4) which practice-management system exports will supply the file, so the columns can be mapped; (5) can one claim legitimately carry the same line twice (for example the same J-code with different NDCs, or separate-line billing of the same service)? The import refuses a repeated procedure code plus modifiers on one claim, and there is no override yet; (6) is it acceptable that a claim's rows must be next to each other in the file (a claim number that comes back after other claims is refused), or do your PM exports interleave claims? Note: the import rate limit (10 per practice per 10 minutes) counts every attempt, refused ones included.</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>The import refuses possible duplicates with no override and creates one claim per Claim number; a wrong assumption blocks real charge files.</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>Answers to the four questions; answers to (5) and (6), and whether 10 attempts per 10 minutes is enough for a billing day.</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>specs/claims.md C2</t>
+        </is>
+      </c>
+      <c r="I84" s="3" t="inlineStr">
+        <is>
+          <t>agent Claude C2 (vigilant-tesla-ps41e9), 2026-09-29</t>
+        </is>
+      </c>
+      <c r="J84" s="3" t="inlineStr">
+        <is>
+          <t>Before the first real practice</t>
+        </is>
+      </c>
+      <c r="K84" s="3" t="inlineStr"/>
+      <c r="L84" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L82"/>
-  <dataValidations count="6">
-    <dataValidation sqref="B10:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>
-    </dataValidation>
+  <autoFilter ref="A1:L84"/>
+  <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>
     </dataValidation>
-    <dataValidation sqref="C10:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"P0,P1,P2,P3"</formula1>
-    </dataValidation>
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
-    </dataValidation>
-    <dataValidation sqref="D10:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Data source,Clarification,Decision,Legal/Compliance,Vendor/Account,Design/Brand,Business"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Data source,Clarification,Decision,Legal/Compliance,Vendor/Account,Design/Brand,Business"</formula1>

</xml_diff>

<commit_message>
docs(claims): split C3 into C3a 837P generation and C3b submission; C3a spec [R-3.10.1, R-4.1, R-7.4.6, R-7.5.1]
Adds the C3a mapping table (837P 005010X222A1 loop and segment per element,
VERIFY marks on every uncertain usage or code value), refusal codes, control
number sequence, synthetic-only guard, and acceptance criteria, approved by
delegated technical authority (2026-09-29). Owner rows OA-085 and OA-086.

AI-Assisted: true
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NY7r13quPdzAWKCKUiLCt2
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$86</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5008,8 +5008,116 @@
       <c r="K84" s="3" t="inlineStr"/>
       <c r="L84" s="3" t="inlineStr"/>
     </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>OA-085</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>Supply the licensed 837P implementation guide (ASC X12 TR3 005010X222A1) and the chosen clearinghouse's 837P companion guide, and answer the C3a claim-level attestations: does the practice hold a signature on file, accept assignment, and hold a release of information for every patient (CLM06 to CLM09)? Confirm the SBR09 claim filing indicator for Medicare Advantage, ERISA self-funded, SMMC, and PIP payers.</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>C3a generates a synthetic (test-indicator T) 837P from knowledge of the guide, not from the guide itself; every row marked VERIFY in specs/claims.md C3a must be cleared before the first real P file, and four payer types are refused until their SBR09 is confirmed.</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>The guide and companion guide (or a written yes/no on each VERIFY row), the four attestation answers, and the SBR09 codes.</t>
+        </is>
+      </c>
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t>specs/claims.md C3a; R-4.1, §8.2</t>
+        </is>
+      </c>
+      <c r="I85" s="3" t="inlineStr">
+        <is>
+          <t>agent Claude C3a (vigilant-tesla-ps41e9), 2026-09-29</t>
+        </is>
+      </c>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>Before C3b</t>
+        </is>
+      </c>
+      <c r="K85" s="3" t="inlineStr"/>
+      <c r="L85" s="3" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>OA-086</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>Decide whether the 837P control numbers (ISA13, GS06, ST02) get a dedicated per-practice sequence table; it needs a GRANT to denialdesk_app, so it needs your sign-off (R-15.9). C3a stores the counter as one practice_settings row (existing table and grant) so it needs no GRANT.</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>The practice_settings row works and is atomic, but it is a general key/value table; a dedicated table with no UPDATE path other than the increment function is easier to audit.</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>Approve or decline a dedicated table and its grant.</t>
+        </is>
+      </c>
+      <c r="H86" s="3" t="inlineStr">
+        <is>
+          <t>specs/claims.md C3a; R-15.9</t>
+        </is>
+      </c>
+      <c r="I86" s="3" t="inlineStr">
+        <is>
+          <t>agent Claude C3a (vigilant-tesla-ps41e9), 2026-09-29</t>
+        </is>
+      </c>
+      <c r="J86" s="3" t="inlineStr">
+        <is>
+          <t>Before C3b</t>
+        </is>
+      </c>
+      <c r="K86" s="3" t="inlineStr"/>
+      <c r="L86" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L84"/>
+  <autoFilter ref="A1:L86"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
docs(integrations): PR #100 review round, ADR 0012, threat model, runbook, spec, owner actions OA-085 to OA-087 [R-7.3.5, R-15.9]
ADR 0012 corrected (abandons are audited by the caller), p_sandbox_only documented, final 0044 + 0045
privilege list. Threat model: unauthenticated invocations and log volume, per-context job secrets,
role separation versus arbitrary SQL, pinned function owner at Azure. Runbook: per-context secrets,
secret-mismatch diagnosis, preview verification of DEPLOY_URL, Background Functions plan and the
deploy log. Owner sheet rebuilt from the base file: OA-085 sign-off (0044 already ran on the preview
branch; preview branches as test databases; roles-reach-shared-database VERIFY), OA-086 secret per
context, OA-087 U.S. regions.

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NY7r13quPdzAWKCKUiLCt2
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$87</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5008,8 +5008,170 @@
       <c r="K84" s="3" t="inlineStr"/>
       <c r="L84" s="3" t="inlineStr"/>
     </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>OA-085</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>Legal/Compliance</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>Sign off (R-15.9) on migrations 0044 and 0045 before they run beyond a local or test database: they create the NOLOGIN role `denialdesk_jobs`, two SECURITY DEFINER functions (`integration_claim_run(uuid)`, `integration_enqueue_due_runs(boolean)`) and their GRANT and REVOKE statements (0045 drops 0044's zero-argument scheduler function and creates its replacement). Every statement is listed verbatim in the PR description, docs/PROJECT_STATE.md and ADR 0012. Also confirm that a Netlify Database preview branch counts as a test database for this rule.</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>Background sync jobs need a database role that can do exactly two things: ask whether a run is a queued run of an active connection (and whose), and queue the 15-minute scheduled runs. The role has no table privilege, `denialdesk_app` is not granted either function, and PUBLIC is revoked first. The functions run as their owner and walk the practices one at a time under each practice's own row-level security policy (no policy or BYPASSRLS is added). Both migrations also check that the integration service-principal row seeded by 0043 is still disabled, has the non-hash password marker, no second-factor secret, the reserved address and no membership, and stop the migration if not. IMPORTANT: 0044 has ALREADY been applied to the Netlify preview database branch of PR #100 (deploy previews get their own database branch); Migration 0043 was in the same position (Netlify previews had applied it when it was approved, OA-076). Netlify has applied 0001 to 0043 to the main preview database; 0044 and 0045 are pending there. ⚠️ VERIFY: roles are cluster-wide in PostgreSQL, so a role created on a preview branch might be visible outside that branch depending on how Netlify Database provisions branches; the agent could not confirm that a role created on a preview branch does not reach the shared pre-production database.</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>Approve, or ask for a different shape (for example the claim as a plain function without the tenant walk, which needs a BYPASSRLS or superuser owner). Say whether preview database branches count as test databases for R-15.9, and whether the ⚠️ VERIFY about roles reaching the shared pre-production database needs checking in the Netlify Database console before merge. Recorded on the PR.</t>
+        </is>
+      </c>
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t>docs/specs/patient-integrations.md (PI2b Jobs, PI3); docs/decisions/0012-background-execution.md; drizzle/0044_patient_integrations_jobs.sql; drizzle/0045_patient_integrations_jobs_review.sql; R-15.9</t>
+        </is>
+      </c>
+      <c r="I85" s="3" t="inlineStr">
+        <is>
+          <t>PI2c jobs builder, 2026-09-29 (revised in the PR #100 review round)</t>
+        </is>
+      </c>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>Before PR #100 is merged (Netlify applies migrations on the next deploy)</t>
+        </is>
+      </c>
+      <c r="K85" s="3" t="n"/>
+      <c r="L85" s="3" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>OA-086</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>Vendor/Account</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>Generate INTEGRATION_JOB_SECRET (at least 32 random bytes, for example `openssl rand -base64 48`) and set it as a functions-only secret in the Netlify site settings, with a DIFFERENT value per deploy context (Production, and separately Deploy Previews and Branch deploys). Confirm the Netlify plan supports Background Functions, and check that the site's own password protection does not block the function URL the app posts jobs to.</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>The secret signs every background sync job (HMAC-SHA256 over the body and a timestamp) and lets the worker refuse forged or replayed ones. Previews run pull-request code, which can read its own environment, so a value shared with production would let a pull request forge jobs against production. Until it is set nothing breaks: Sync now keeps running in the request as before (only where synthetic data is allowed), and the worker and the 15-minute scheduled function refuse to run. Once it is set, Sync now queues a job by posting to this deploy's own `/.netlify/functions/integration-sync-background`, and the site is behind Netlify password protection. If that protection also covers function URLs the post is refused (a 401 from Netlify) and Sync now reports that the sync could not be started; the fix would then be an exemption for that path or a basic-auth header, a small follow-up. Background Functions (the `-background` suffix) need a plan that includes them. Scheduled functions run only on the published (production) deploy, not on deploy previews. Whether `DEPLOY_URL` or `URL` exist at function and server runtime is also unverified (the runbook lists how to check). Never commit the value; production keeps it in Key Vault.</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>Confirmation the secret is set for functions only (not the build or the client), that Production and the preview contexts hold different values, and that the plan supports Background Functions; then, after the next deploy, press Sync now on the pre-production sandbox connection and confirm it says the sync was queued and a run appears in Sync history, and that a scheduled run appears within 15 minutes; and that the deploy log lists both functions. Tell the agent if the press says it could not be started.</t>
+        </is>
+      </c>
+      <c r="H86" s="3" t="inlineStr">
+        <is>
+          <t>docs/specs/patient-integrations.md PI2b Jobs, PI3; docs/decisions/0012-background-execution.md; docs/runbooks/netlify.md; R-7.3.5</t>
+        </is>
+      </c>
+      <c r="I86" s="3" t="inlineStr">
+        <is>
+          <t>PI2c jobs builder, 2026-09-29 (revised in the PR #100 review round)</t>
+        </is>
+      </c>
+      <c r="J86" s="3" t="inlineStr">
+        <is>
+          <t>Before the first background sync on Netlify</t>
+        </is>
+      </c>
+      <c r="K86" s="3" t="n"/>
+      <c r="L86" s="3" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>OA-087</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>Legal/Compliance</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>Confirm that the Netlify Functions region and the Netlify Database region for this site are in the United States, and record where you checked.</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>ADR 0003 leaves this as ⚠️ VERIFY: Netlify is not the HIPAA host and its functions are not restricted to U.S. regions the way the Azure landing zone will be. Until now the Netlify code ran only when a person pressed a button on synthetic data. The 15-minute scheduled function and the background worker now process data unattended there, so Fla. Stat. § 408.051(3) residency should be confirmed even though pre-production holds synthetic data only (CLAUDE.md non-negotiable 3).</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>The region shown in the Netlify site settings for Functions and for the database, or a statement that either cannot be confirmed (then the scheduler should stay off until it can).</t>
+        </is>
+      </c>
+      <c r="H87" s="3" t="inlineStr">
+        <is>
+          <t>docs/decisions/0003-netlify-preproduction.md; docs/decisions/0012-background-execution.md; CLAUDE.md non-negotiable 3</t>
+        </is>
+      </c>
+      <c r="I87" s="3" t="inlineStr">
+        <is>
+          <t>PI2c jobs builder, 2026-09-29 (PR #100 review round)</t>
+        </is>
+      </c>
+      <c r="J87" s="3" t="inlineStr">
+        <is>
+          <t>Before enabling the scheduled function on Netlify</t>
+        </is>
+      </c>
+      <c r="K87" s="3" t="n"/>
+      <c r="L87" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L84"/>
+  <autoFilter ref="A1:L87"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
fix(patients): member-ID review round: unmapped wording, NULL-payer tests, OA-085 [R-5.1.2, R-7.5.1, R-11.1]
- Label reads "Not on file for this claim's payer" (en/es/pt) so it is also true for
  synced patients with unmapped coverage (no primary payer).
- Reveal actions answer "Not found" when no member ID is on file (empty last four),
  before the payer check.
- Integration test: deterministic fixtures, and cases for no payer mapped and no member
  ID on file, exercising the SQL fragments' NULL handling.
- Stale "shown the same as self-pay" comments updated.
- OA-085: owner decision on auditing refused reveal attempts.

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AV7pay23TPhuytCLjTGZac
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$85</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5008,8 +5008,62 @@
       <c r="K84" s="3" t="inlineStr"/>
       <c r="L84" s="3" t="inlineStr"/>
     </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>OA-085</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>Legal/Compliance</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>Decide whether refused reveal attempts (member ID on another payer's claim, locked custom fields, wrong role) should write their own audit event such as patient.member_id_reveal_refused.</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>Today a refused reveal writes no audit event (nothing is decrypted), unlike refused charge imports and step-ups; auditing it would give SIEM alerting (R-7.5.3) a signal for crafted requests.</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>Yes/no, and if yes which refusals; the agent adds an IDs-only refusal event and tests.</t>
+        </is>
+      </c>
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t>R-5.1.2, R-7.5.1, R-7.5.3; specs/denial-queue.md</t>
+        </is>
+      </c>
+      <c r="I85" s="3" t="inlineStr">
+        <is>
+          <t>Claude scheduled review 2026-09-29</t>
+        </is>
+      </c>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>Before Azure cutover</t>
+        </is>
+      </c>
+      <c r="K85" s="3" t="inlineStr"/>
+      <c r="L85" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L84"/>
+  <autoFilter ref="A1:L85"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
feat(integrations): signed background sync jobs, 15-minute schedule, repeated-failure error (PI2c/PI3) [R-5.1.2, R-7.2.4, R-7.5.1, R-15.9] (#100)
HMAC-signed {runId} jobs to a Netlify Background Function worker; 15-minute
scheduled enqueue (sandbox-only until PI4) with lease abandon and audit; Sync now
posts a job; three consecutive failed runs set the connection to error.
Migrations 0044/0045 add NOLOGIN role denialdesk_jobs and two SECURITY DEFINER
functions — owner R-15.9 sign-off recorded 2026-09-29 (OA-085).

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NY7r13quPdzAWKCKUiLCt2
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$87</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5008,8 +5008,170 @@
       <c r="K84" s="3" t="inlineStr"/>
       <c r="L84" s="3" t="inlineStr"/>
     </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>OA-085</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>Legal/Compliance</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>Sign off (R-15.9) on migrations 0044 and 0045 before they run beyond a local or test database: they create the NOLOGIN role `denialdesk_jobs`, two SECURITY DEFINER functions (`integration_claim_run(uuid)`, `integration_enqueue_due_runs(boolean)`) and their GRANT and REVOKE statements (0045 drops 0044's zero-argument scheduler function and creates its replacement). Every statement is listed verbatim in the PR description, docs/PROJECT_STATE.md and ADR 0012. Also confirm that a Netlify Database preview branch counts as a test database for this rule.</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>Background sync jobs need a database role that can do exactly two things: ask whether a run is a queued run of an active connection (and whose), and queue the 15-minute scheduled runs. The role has no table privilege, `denialdesk_app` is not granted either function, and PUBLIC is revoked first. The functions run as their owner and walk the practices one at a time under each practice's own row-level security policy (no policy or BYPASSRLS is added). Both migrations also check that the integration service-principal row seeded by 0043 is still disabled, has the non-hash password marker, no second-factor secret, the reserved address and no membership, and stop the migration if not. IMPORTANT: 0044 has ALREADY been applied to the Netlify preview database branch of PR #100 (deploy previews get their own database branch); Migration 0043 was in the same position (Netlify previews had applied it when it was approved, OA-076). Netlify has applied 0001 to 0043 to the main preview database; 0044 and 0045 are pending there. ⚠️ VERIFY: roles are cluster-wide in PostgreSQL, so a role created on a preview branch might be visible outside that branch depending on how Netlify Database provisions branches; the agent could not confirm that a role created on a preview branch does not reach the shared pre-production database. ⚠️ VERIFY: that Netlify Database applies each migration.sql in a single transaction. If it does not, PUBLIC briefly holds EXECUTE on a new function between its CREATE FUNCTION and the REVOKE that follows it (in 0044 and 0045); the functions only return identifiers and check their caller's tenant setting, but the window should be known. The agent could not confirm how Netlify runs a migration file.</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>Approve, or ask for a different shape (for example the claim as a plain function without the tenant walk, which needs a BYPASSRLS or superuser owner). Say whether preview database branches count as test databases for R-15.9, and whether the ⚠️ VERIFY about roles reaching the shared pre-production database needs checking in the Netlify Database console before merge. Recorded on the PR. Also whether Netlify Database runs each migration file in one transaction.</t>
+        </is>
+      </c>
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t>docs/specs/patient-integrations.md (PI2b Jobs, PI3); docs/decisions/0012-background-execution.md; drizzle/0044_patient_integrations_jobs.sql; drizzle/0045_patient_integrations_jobs_review.sql; R-15.9</t>
+        </is>
+      </c>
+      <c r="I85" s="3" t="inlineStr">
+        <is>
+          <t>PI2c jobs builder, 2026-09-29 (revised in the PR #100 review round)</t>
+        </is>
+      </c>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>Before PR #100 is merged (Netlify applies migrations on the next deploy)</t>
+        </is>
+      </c>
+      <c r="K85" s="3" t="n"/>
+      <c r="L85" s="3" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>OA-086</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>Vendor/Account</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>Generate INTEGRATION_JOB_SECRET (at least 32 random bytes, for example `openssl rand -base64 48`) and set it as a functions-only secret in the Netlify site settings, with a DIFFERENT value per deploy context (Production, and separately Deploy Previews and Branch deploys). Confirm the Netlify plan supports Background Functions, and check that the site's own password protection does not block the function URL the app posts jobs to.</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>The secret signs every background sync job (HMAC-SHA256 over the body and a timestamp) and lets the worker refuse forged or replayed ones. Previews run pull-request code, which can read its own environment, so a value shared with production would let a pull request forge jobs against production. Until it is set nothing breaks: Sync now keeps running in the request as before (only where synthetic data is allowed), and the worker and the 15-minute scheduled function refuse to run. Once it is set, Sync now queues a job by posting to this deploy's own `/.netlify/functions/integration-sync-background`, and the site is behind Netlify password protection. If that protection also covers function URLs the post is refused (a 401 from Netlify) and Sync now reports that the sync could not be started; the fix would then be an exemption for that path or a basic-auth header, a small follow-up. Background Functions (the `-background` suffix) need a plan that includes them. Scheduled functions run only on the published (production) deploy, not on deploy previews. Whether `DEPLOY_URL` or `URL` exist at function and server runtime is also unverified (the runbook lists how to check). Never commit the value; production keeps it in Key Vault.</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>Confirmation the secret is set for functions only (not the build or the client), that Production and the preview contexts hold different values, and that the plan supports Background Functions; then, after the next deploy, press Sync now on the pre-production sandbox connection and confirm it says the sync was queued and a run appears in Sync history, and that a scheduled run appears within 15 minutes; and that the deploy log lists both functions. Tell the agent if the press says it could not be started.</t>
+        </is>
+      </c>
+      <c r="H86" s="3" t="inlineStr">
+        <is>
+          <t>docs/specs/patient-integrations.md PI2b Jobs, PI3; docs/decisions/0012-background-execution.md; docs/runbooks/netlify.md; R-7.3.5</t>
+        </is>
+      </c>
+      <c r="I86" s="3" t="inlineStr">
+        <is>
+          <t>PI2c jobs builder, 2026-09-29 (revised in the PR #100 review round)</t>
+        </is>
+      </c>
+      <c r="J86" s="3" t="inlineStr">
+        <is>
+          <t>Before the first background sync on Netlify</t>
+        </is>
+      </c>
+      <c r="K86" s="3" t="n"/>
+      <c r="L86" s="3" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>OA-087</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>Legal/Compliance</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>Confirm that the Netlify Functions region and the Netlify Database region for this site are in the United States, and record where you checked.</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>ADR 0003 leaves this as ⚠️ VERIFY: Netlify is not the HIPAA host and its functions are not restricted to U.S. regions the way the Azure landing zone will be. Until now the Netlify code ran only when a person pressed a button on synthetic data. The 15-minute scheduled function and the background worker now process data unattended there, so Fla. Stat. § 408.051(3) residency should be confirmed even though pre-production holds synthetic data only (CLAUDE.md non-negotiable 3).</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>The region shown in the Netlify site settings for Functions and for the database, or a statement that either cannot be confirmed (then the scheduler should stay off until it can).</t>
+        </is>
+      </c>
+      <c r="H87" s="3" t="inlineStr">
+        <is>
+          <t>docs/decisions/0003-netlify-preproduction.md; docs/decisions/0012-background-execution.md; CLAUDE.md non-negotiable 3</t>
+        </is>
+      </c>
+      <c r="I87" s="3" t="inlineStr">
+        <is>
+          <t>PI2c jobs builder, 2026-09-29 (PR #100 review round)</t>
+        </is>
+      </c>
+      <c r="J87" s="3" t="inlineStr">
+        <is>
+          <t>Before enabling the scheduled function on Netlify</t>
+        </is>
+      </c>
+      <c r="K87" s="3" t="n"/>
+      <c r="L87" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L84"/>
+  <autoFilter ref="A1:L87"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
feat(claims): C3a 837P (005010X222A1) generation, validation and synthetic download [§4.1, §8.2, R-3.10.1, R-7.5.1] (#102)
Pure 837P generator (codes copied exactly; ICD-10 decimal dropped as X12
representation only), claim service with coverage guards before any decrypt,
field-encrypted provider TIN, per-practice control numbers, synthetic-only
(ISA15=T), masked preview and browser-built download, audited. Migration 0046
adds nullable billing columns only. Pre-C3b blockers recorded (sensitive
diagnoses, pointer persistence, attestations, OA-091).

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NY7r13quPdzAWKCKUiLCt2
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$91</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L88"/>
+  <dimension ref="A1:L91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5224,8 +5224,170 @@
       <c r="K88" s="3" t="n"/>
       <c r="L88" s="3" t="n"/>
     </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>OA-089</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>Supply the licensed 837P implementation guide (ASC X12 TR3 005010X222A1) and the chosen clearinghouse's 837P companion guide, and answer the C3a claim-level attestations: does the practice hold a signature on file, accept assignment, and hold a release of information for every patient (CLM06 to CLM09)? Confirm the SBR09 claim filing indicator for Medicare Advantage, ERISA self-funded, SMMC, and PIP payers.</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>C3a generates a synthetic (test-indicator T) 837P from knowledge of the guide, not from the guide itself; every row marked VERIFY in specs/claims.md C3a must be cleared before the first real P file, and four payer types are refused until their SBR09 is confirmed.</t>
+        </is>
+      </c>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>The guide and companion guide (or a written yes/no on each VERIFY row), the four attestation answers, and the SBR09 codes.</t>
+        </is>
+      </c>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>specs/claims.md C3a; R-4.1, §8.2</t>
+        </is>
+      </c>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
+          <t>agent Claude C3a (vigilant-tesla-ps41e9), 2026-09-29</t>
+        </is>
+      </c>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>Before C3b</t>
+        </is>
+      </c>
+      <c r="K89" s="3" t="n"/>
+      <c r="L89" s="3" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>OA-090</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>Decide whether the 837P control numbers (ISA13, GS06, ST02) get a dedicated per-practice sequence table; it needs a GRANT to denialdesk_app, so it needs your sign-off (R-15.9). C3a stores the counter as one practice_settings row (existing table and grant) so it needs no GRANT.</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>The practice_settings row works and is atomic, but it is a general key/value table; a dedicated table with no UPDATE path other than the increment function is easier to audit.</t>
+        </is>
+      </c>
+      <c r="G90" s="3" t="inlineStr">
+        <is>
+          <t>Approve or decline a dedicated table and its grant.</t>
+        </is>
+      </c>
+      <c r="H90" s="3" t="inlineStr">
+        <is>
+          <t>specs/claims.md C3a; R-15.9</t>
+        </is>
+      </c>
+      <c r="I90" s="3" t="inlineStr">
+        <is>
+          <t>agent Claude C3a (vigilant-tesla-ps41e9), 2026-09-29</t>
+        </is>
+      </c>
+      <c r="J90" s="3" t="inlineStr">
+        <is>
+          <t>Before C3b</t>
+        </is>
+      </c>
+      <c r="K90" s="3" t="n"/>
+      <c r="L90" s="3" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>OA-091</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Legal/Compliance</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>Answer three C3a compliance questions with counsel: (1) does DenialDesk become a HIPAA health care clearinghouse by generating standard transactions (837P) for practices, and what follows; (2) how are 42 CFR Part 2 consent and sensitivity-tagged diagnoses handled on outgoing claims; (3) may real claim files ever be downloaded to a person's device, or only sent to the clearinghouse.</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>C3a already builds and offers a download of the 837P (synthetic only). These answers gate C3b and any real claim.</t>
+        </is>
+      </c>
+      <c r="G91" s="3" t="inlineStr">
+        <is>
+          <t>Counsel answers or a decision on each of the three.</t>
+        </is>
+      </c>
+      <c r="H91" s="3" t="inlineStr">
+        <is>
+          <t>specs/claims.md C3a; R-3.5.1, R-3.5.2, R-4.1</t>
+        </is>
+      </c>
+      <c r="I91" s="3" t="inlineStr">
+        <is>
+          <t>agent Claude C3a (vigilant-tesla-ps41e9), 2026-09-29</t>
+        </is>
+      </c>
+      <c r="J91" s="3" t="inlineStr">
+        <is>
+          <t>Before C3b</t>
+        </is>
+      </c>
+      <c r="K91" s="3" t="n"/>
+      <c r="L91" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L87"/>
+  <autoFilter ref="A1:L91"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
docs(crypto): close reviewer and compliance follow-ups on the TIN plan [R-7.3.3]
- PR 1/2: CI and the Playwright preview server set FIELD_LEGACY_V1_READ=on until PR 5, since
  writers and fixtures still write v1 until PR 3.
- PR 2 keeps the test key on decryptProviderTin until PR 3; PR 3 drops the vacuous no-AAD test.
- Seed tenant allowed as the member ID AAD scope in seedPractice.
- TIN integrity event names the provider record; residual risks cover pre-PR 2 837P failures
  and same-row replay for every column; TIN classification cites REQUIREMENTS §9.1.
- Spec question 12 (refuse v1 provider TINs in production), tracked under OA-078.

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QCaBhuvNddsqynubD6Mpxq
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -4653,7 +4653,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Approve an ADR and a re-encryption migration to bind field-level encryption to its record: today the encrypted member ID (and every other encrypted field) has no additional authenticated data (AAD) tying the ciphertext to its row and practice. Proposed design: ADR 0011 (docs/decisions/0011-field-encryption-aad-envelope-v2.md, PR #97) with spec docs/specs/field-encryption-aad.md; also answer spec questions 2-5: run the re-encryption job on pre-production or wipe and re-seed (security review recommends re-seed); who confirms the legacy cut-off; confirm Azure production starts empty; whether the pre-production FIELD_ENCRYPTION_KEY was ever changed.</t>
+          <t>Approve an ADR and a re-encryption migration to bind field-level encryption to its record: today the encrypted member ID (and every other encrypted field) has no additional authenticated data (AAD) tying the ciphertext to its row and practice. Proposed design: ADR 0011 (docs/decisions/0011-field-encryption-aad-envelope-v2.md, PR #97) with spec docs/specs/field-encryption-aad.md; also answer spec questions 2-5 and 12: run the re-encryption job on pre-production or wipe and re-seed (security review recommends re-seed); who confirms the legacy cut-off; confirm Azure production starts empty; whether the pre-production FIELD_ENCRYPTION_KEY was ever changed; whether production refuses legacy (v1) provider TINs.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -4663,7 +4663,7 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Approval of ADR 0011 (or requested changes) and the timing; answers to spec questions 2-5.</t>
+          <t>Approval of ADR 0011 (or requested changes) and the timing; answers to spec questions 2-5 and 12.</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs(owner): add OA-093 to OA-096 for appeal letter decisions [R-7.11.2]
Spanish/Portuguese letter templates and template history, full member ID on the export,
a payer address field, and who may attest / whether submission needs an attestation.

AI-Assisted: true
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NY7r13quPdzAWKCKUiLCt2
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$96</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L92"/>
+  <dimension ref="A1:L96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5440,8 +5440,224 @@
       <c r="K92" s="3" t="n"/>
       <c r="L92" s="3" t="n"/>
     </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>OA-093</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>Clarification</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>Decide whether Spanish and Portuguese payer-facing appeal letter templates are needed, and whether template edits need their own version history.</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>A letter goes to the payer, so A2 ships English templates only (the UI around them is en/es/pt). A template history table would need a new GRANT (R-15.9).</t>
+        </is>
+      </c>
+      <c r="G93" s="3" t="inlineStr">
+        <is>
+          <t>Yes/no per language; yes/no for template history.</t>
+        </is>
+      </c>
+      <c r="H93" s="3" t="inlineStr">
+        <is>
+          <t>specs/appeals.md A2; R-7.11.2</t>
+        </is>
+      </c>
+      <c r="I93" s="3" t="inlineStr">
+        <is>
+          <t>agent Claude A2 (vigilant-tesla-ps41e9), 2026-09-29</t>
+        </is>
+      </c>
+      <c r="J93" s="3" t="inlineStr">
+        <is>
+          <t>Before A3</t>
+        </is>
+      </c>
+      <c r="K93" s="3" t="inlineStr"/>
+      <c r="L93" s="3" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>OA-094</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>Decide whether an exported appeal letter may show the full member ID (decrypted at print time, audited) or only the last four characters.</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>Payers often need the full ID. A2 masks it (minimum necessary, HC-3.3; field-level encryption, R-7.3.3) and the biller types the full ID after the audited reveal on the appeal page.</t>
+        </is>
+      </c>
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>Keep masked, or allow the full ID on the print view only.</t>
+        </is>
+      </c>
+      <c r="H94" s="3" t="inlineStr">
+        <is>
+          <t>specs/appeals.md A2; HC-3.3; R-7.3.3</t>
+        </is>
+      </c>
+      <c r="I94" s="3" t="inlineStr">
+        <is>
+          <t>agent Claude A2 (vigilant-tesla-ps41e9), 2026-09-29</t>
+        </is>
+      </c>
+      <c r="J94" s="3" t="inlineStr">
+        <is>
+          <t>Before real data</t>
+        </is>
+      </c>
+      <c r="K94" s="3" t="inlineStr"/>
+      <c r="L94" s="3" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>OA-095</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>Decide where a payer's appeals mailing address and fax number should live so letters can merge them (a new column on payers, or a per-appeal field).</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>The payers table has no address column, so starter letters carry a fill-in placeholder for it. A new column needs a migration.</t>
+        </is>
+      </c>
+      <c r="G95" s="3" t="inlineStr">
+        <is>
+          <t>Choice of location and where the addresses come from.</t>
+        </is>
+      </c>
+      <c r="H95" s="3" t="inlineStr">
+        <is>
+          <t>specs/appeals.md A2; specs/payer-catalog.md</t>
+        </is>
+      </c>
+      <c r="I95" s="3" t="inlineStr">
+        <is>
+          <t>agent Claude A2 (vigilant-tesla-ps41e9), 2026-09-29</t>
+        </is>
+      </c>
+      <c r="J95" s="3" t="inlineStr">
+        <is>
+          <t>Before A3</t>
+        </is>
+      </c>
+      <c r="K95" s="3" t="inlineStr"/>
+      <c r="L95" s="3" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>OA-096</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>Confirm who may attest and export appeal letters (built: admin, manager, specialist; compliance read-only), whether a second person must review a letter the author wrote, and whether recording a submission should require an attestation.</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>R-7.11.2 requires a named user to approve before anything reaches a payer. A2 blocks export without an attestation but does not require four eyes or gate 'record submission'.</t>
+        </is>
+      </c>
+      <c r="G96" s="3" t="inlineStr">
+        <is>
+          <t>A decision on each of the three.</t>
+        </is>
+      </c>
+      <c r="H96" s="3" t="inlineStr">
+        <is>
+          <t>specs/appeals.md A2; R-7.11.2, R-5.1.2</t>
+        </is>
+      </c>
+      <c r="I96" s="3" t="inlineStr">
+        <is>
+          <t>agent Claude A2 (vigilant-tesla-ps41e9), 2026-09-29</t>
+        </is>
+      </c>
+      <c r="J96" s="3" t="inlineStr">
+        <is>
+          <t>Before A3</t>
+        </is>
+      </c>
+      <c r="K96" s="3" t="inlineStr"/>
+      <c r="L96" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L91"/>
+  <autoFilter ref="A1:L96"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
fix(settings): billing review round - TIN change semantics, list status, tests [R-7.2.2, R-7.3.3, R-7.5.1]
- A type-only TIN change sets the type without decrypting (the AAD excludes the type);
  re-typing the stored TIN is no change (no write, no audit).
- List flags a ZIP without nine digits and an unreadable TIN, names the missing fields,
  and audits the readability check; view audit marks tin_unreadable.
- Form clears the TIN after submit; bound failures show field errors; both forms alike.
- Tests: fix save-resends-TIN audit flake, event ordering, metadata-only POS check,
  never-issued SSN area for the second synthetic TIN, drop a meaningless test.
- Comments and spec: step-up targets, provider-tin readers, open question OA-097, HC-4.2 gap.

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NY7r13quPdzAWKCKUiLCt2
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$94</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L93"/>
+  <dimension ref="A1:L94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5494,8 +5494,62 @@
       <c r="K93" s="3" t="n"/>
       <c r="L93" s="3" t="n"/>
     </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>OA-097</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>Decide whether changing a provider's billing name or address (not only the TIN) should also require a fresh step-up MFA on Settings &gt; Billing.</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>They go on every claim, so a wrong address misdirects payment. C3a-S asks for the step-up only when the TIN is set or changed, to keep the page usable.</t>
+        </is>
+      </c>
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>Yes or no, and if yes which fields.</t>
+        </is>
+      </c>
+      <c r="H94" s="3" t="inlineStr">
+        <is>
+          <t>specs/claims.md C3a-S; R-7.2.2, HC-4.2</t>
+        </is>
+      </c>
+      <c r="I94" s="3" t="inlineStr">
+        <is>
+          <t>agent Claude C3a-S (vigilant-tesla-ps41e9), 2026-09-29</t>
+        </is>
+      </c>
+      <c r="J94" s="3" t="inlineStr">
+        <is>
+          <t>Before launch</t>
+        </is>
+      </c>
+      <c r="K94" s="3" t="n"/>
+      <c r="L94" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L93"/>
+  <autoFilter ref="A1:L94"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
feat(settings): provider billing details and place of service page (C3a-S) [R-7.2.2, R-7.3.3, R-7.5.1, R-3.10.1] (#104)
Settings > Billing: admin page for provider billing name, address, TIN type and
write-only TIN (field-encrypted, step-up MFA to set or change, last four only,
decrypts audited), and location place of service. X12-safe validation matching
the 0046 CHECKs; column-name-only audit; no migration, no GRANT.

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NY7r13quPdzAWKCKUiLCt2
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$97</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5389,7 +5389,7 @@
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>OA-101</t>
+          <t>OA-092</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
@@ -5404,37 +5404,37 @@
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Legal/Compliance</t>
+          <t>Data source</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>Decide whether local development may keep Next.js's unavoidable 'next dev' update check (it asks registry.npmjs.org for newer Next.js versions; no opt-out in 16.3.6) under a written, time-boxed exception ADR signed by the Security and Privacy Officers (HC §0), or keep SC-A2.6 tracked as a known gap.</t>
+          <t>Supply the CMS place of service (POS) code set, and tell us which codes the practice bills from each location, so the Billing settings page can check a code against the real list. Today it checks only that the code is two digits.</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>SC-A2.6 bans update checks; everything else that phones home is now off. No PHI is involved (local development holds synthetic data only).</t>
+          <t>A wrong POS code changes how a payer prices and pays the claim. The page (specs/claims.md C3a-S) and the 837P generator check the format only, and DenialDesk does not state what a code means without a source.</t>
         </is>
       </c>
       <c r="G92" s="3" t="inlineStr">
         <is>
-          <t>Accept (officers sign an exception ADR the agent drafts) or keep tracked.</t>
+          <t>The CMS POS code set file (or the link the practice uses) and, per location, the code it bills with.</t>
         </is>
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>SC-A2.6; HC §0; PR #96</t>
+          <t>specs/claims.md C3a-S; R-4.1</t>
         </is>
       </c>
       <c r="I92" s="3" t="inlineStr">
         <is>
-          <t>SC gap PRs session 2026-09-29</t>
+          <t>agent Claude C3a-S (vigilant-tesla-ps41e9), 2026-09-29</t>
         </is>
       </c>
       <c r="J92" s="3" t="inlineStr">
         <is>
-          <t>Before the first real practice</t>
+          <t>Before C3b</t>
         </is>
       </c>
       <c r="K92" s="3" t="n"/>
@@ -5443,7 +5443,7 @@
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>OA-102</t>
+          <t>OA-097</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -5463,32 +5463,32 @@
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>Approve a separate RATE_LIMIT_HASH_KEY so src/lib/rate-limit.ts stops reusing FIELD_ENCRYPTION_KEY as a hash salt (spec question 6).</t>
+          <t>Decide whether changing a provider's billing name or address (not only the TIN) should also require a fresh step-up MFA on Settings &gt; Billing.</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>One key per purpose; rotating the field key must not reset rate-limit windows.</t>
+          <t>They go on every claim, so a wrong address misdirects payment. C3a-S asks for the step-up only when the TIN is set or changed, to keep the page usable.</t>
         </is>
       </c>
       <c r="G93" s="3" t="inlineStr">
         <is>
-          <t>Yes/no; if yes the agent adds the variable in a follow-up PR (never the value in the sheet).</t>
+          <t>Yes or no, and if yes which fields.</t>
         </is>
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>SC-B7.1; R-7.3.4; docs/specs/field-encryption-aad.md</t>
+          <t>specs/claims.md C3a-S; R-7.2.2, HC-4.2</t>
         </is>
       </c>
       <c r="I93" s="3" t="inlineStr">
         <is>
-          <t>SC-B7.1 AAD plan session 2026-09-28</t>
+          <t>agent Claude C3a-S (vigilant-tesla-ps41e9), 2026-09-29</t>
         </is>
       </c>
       <c r="J93" s="3" t="inlineStr">
         <is>
-          <t>Before the first key rotation</t>
+          <t>Before launch</t>
         </is>
       </c>
       <c r="K93" s="3" t="n"/>
@@ -5497,7 +5497,7 @@
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>OA-103</t>
+          <t>OA-101</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
@@ -5507,42 +5507,42 @@
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Legal/Compliance</t>
         </is>
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Decide the ADR 0011 follow-ups (spec questions 7-10): keep retired keys decrypt-only for append-only custom-field history and synced patients or approve a re-encryption path (R-15.9); key retirement: backup and point-in-time retention periods, no key destruction until legal hold exists, and Security plus Privacy Officer sign-off to destroy a key; run one pre-production key-rotation drill after the cut-off; whether an 835 or find-by-member-ID feature gets a tenant-keyed blind index.</t>
+          <t>Decide whether local development may keep Next.js's unavoidable 'next dev' update check (it asks registry.npmjs.org for newer Next.js versions; no opt-out in 16.3.6) under a written, time-boxed exception ADR signed by the Security and Privacy Officers (HC §0), or keep SC-A2.6 tracked as a known gap.</t>
         </is>
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>Shapes the Azure-cutover key rotation ADR and any member-ID matching feature.</t>
+          <t>SC-A2.6 bans update checks; everything else that phones home is now off. No PHI is involved (local development holds synthetic data only).</t>
         </is>
       </c>
       <c r="G94" s="3" t="inlineStr">
         <is>
-          <t>An answer to each of the four (rotation path, key retirement policy, drill, blind index); the rotation parts can wait for the cutover ADR.</t>
+          <t>Accept (officers sign an exception ADR the agent drafts) or keep tracked.</t>
         </is>
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>SC-B7.1; R-7.3.4; R-15.9; docs/specs/field-encryption-aad.md</t>
+          <t>SC-A2.6; HC §0; PR #96</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
         <is>
-          <t>SC-B7.1 AAD plan session 2026-09-28</t>
+          <t>SC gap PRs session 2026-09-29</t>
         </is>
       </c>
       <c r="J94" s="3" t="inlineStr">
         <is>
-          <t>Azure cutover</t>
+          <t>Before the first real practice</t>
         </is>
       </c>
       <c r="K94" s="3" t="n"/>
@@ -5551,7 +5551,7 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>OA-104</t>
+          <t>OA-102</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -5571,39 +5571,147 @@
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>Decide whether rcm_claim_lines.account_number (the practice's patient account number in revenue-cycle files) is field-encrypted like member IDs.</t>
+          <t>Approve a separate RATE_LIMIT_HASH_KEY so src/lib/rate-limit.ts stops reusing FIELD_ENCRYPTION_KEY as a hash salt (spec question 6).</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>HC-7.3/R-7.3.3 list only SSN, MBI, member IDs, and bank data, so plaintext breaks no MUST rule today; it is still an HC-1.1 identifier protected only by at-rest encryption and RLS.</t>
+          <t>One key per purpose; rotating the field key must not reset rate-limit windows.</t>
         </is>
       </c>
       <c r="G95" s="3" t="inlineStr">
         <is>
-          <t>Yes/no from the Security and Privacy Officers; if yes, the agent adds it to the ADR 0011 build.</t>
+          <t>Yes/no; if yes the agent adds the variable in a follow-up PR (never the value in the sheet).</t>
         </is>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>SC-B7.1; HC-1.1; HC-7.3; ADR 0011; docs/specs/field-encryption-aad.md</t>
+          <t>SC-B7.1; R-7.3.4; docs/specs/field-encryption-aad.md</t>
         </is>
       </c>
       <c r="I95" s="3" t="inlineStr">
         <is>
-          <t>SC-B7.1 AAD plan session 2026-09-29</t>
+          <t>SC-B7.1 AAD plan session 2026-09-28</t>
         </is>
       </c>
       <c r="J95" s="3" t="inlineStr">
         <is>
-          <t>Before the first real practice</t>
+          <t>Before the first key rotation</t>
         </is>
       </c>
       <c r="K95" s="3" t="n"/>
       <c r="L95" s="3" t="n"/>
     </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>OA-103</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>Decide the ADR 0011 follow-ups (spec questions 7-10): keep retired keys decrypt-only for append-only custom-field history and synced patients or approve a re-encryption path (R-15.9); key retirement: backup and point-in-time retention periods, no key destruction until legal hold exists, and Security plus Privacy Officer sign-off to destroy a key; run one pre-production key-rotation drill after the cut-off; whether an 835 or find-by-member-ID feature gets a tenant-keyed blind index.</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>Shapes the Azure-cutover key rotation ADR and any member-ID matching feature.</t>
+        </is>
+      </c>
+      <c r="G96" s="3" t="inlineStr">
+        <is>
+          <t>An answer to each of the four (rotation path, key retirement policy, drill, blind index); the rotation parts can wait for the cutover ADR.</t>
+        </is>
+      </c>
+      <c r="H96" s="3" t="inlineStr">
+        <is>
+          <t>SC-B7.1; R-7.3.4; R-15.9; docs/specs/field-encryption-aad.md</t>
+        </is>
+      </c>
+      <c r="I96" s="3" t="inlineStr">
+        <is>
+          <t>SC-B7.1 AAD plan session 2026-09-28</t>
+        </is>
+      </c>
+      <c r="J96" s="3" t="inlineStr">
+        <is>
+          <t>Azure cutover</t>
+        </is>
+      </c>
+      <c r="K96" s="3" t="n"/>
+      <c r="L96" s="3" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>OA-104</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>Decide whether rcm_claim_lines.account_number (the practice's patient account number in revenue-cycle files) is field-encrypted like member IDs.</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>HC-7.3/R-7.3.3 list only SSN, MBI, member IDs, and bank data, so plaintext breaks no MUST rule today; it is still an HC-1.1 identifier protected only by at-rest encryption and RLS.</t>
+        </is>
+      </c>
+      <c r="G97" s="3" t="inlineStr">
+        <is>
+          <t>Yes/no from the Security and Privacy Officers; if yes, the agent adds it to the ADR 0011 build.</t>
+        </is>
+      </c>
+      <c r="H97" s="3" t="inlineStr">
+        <is>
+          <t>SC-B7.1; HC-1.1; HC-7.3; ADR 0011; docs/specs/field-encryption-aad.md</t>
+        </is>
+      </c>
+      <c r="I97" s="3" t="inlineStr">
+        <is>
+          <t>SC-B7.1 AAD plan session 2026-09-29</t>
+        </is>
+      </c>
+      <c r="J97" s="3" t="inlineStr">
+        <is>
+          <t>Before the first real practice</t>
+        </is>
+      </c>
+      <c r="K97" s="3" t="n"/>
+      <c r="L97" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L95"/>
+  <autoFilter ref="A1:L97"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
docs(data-model): address PR #107 review findings on ADR 0013 and HC-3.x [§9.2]
- ADR 0013 back to Proposed until the owner approves the PR in writing (HC-13.2, OA-106)
- HC-3.5: all HC-1.1 identifiers, subscriber/guarantor home open, claim-scoped IDs,
  no identity in custom fields; HC-3.6 scoped to specs from 2026-09-29
- HC-3.7 follows §9.2 retention, legal hold, and disposal; early disposal to counsel (OA-105)
- HC-3.8 cites Safe Harbor; cross-practice analytics split into HC-3.9 (follows HC-1.4)
- Known gaps: HC-3.6 backlog, retention purge; corrected rcm_claim_lines row and date
- ADR: requirement IDs, encounter audit/FK/backfill needs, claims-column drift, subscriber identity
- compliance-checker checks HC-3.5/3.6; stale field-encryption-aad note updated

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TUv9KsDzYW8LQ1t8PjnRcr
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Action Items" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action Items'!$A$1:$L$99</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L97"/>
+  <dimension ref="A1:L99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5710,8 +5710,116 @@
       <c r="K97" s="3" t="n"/>
       <c r="L97" s="3" t="n"/>
     </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>OA-105</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>Legal/Compliance</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>Decide with counsel whether appeal attachments (clinical records) may be disposed of after sending, keeping a manifest and hash, or must be kept for the appeal-record retention period.</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>HC-3.7 (ADR 0013) keeps them for the full appeal-record period until answered; affects storage of PHI in appeal packets (A5).</t>
+        </is>
+      </c>
+      <c r="G98" s="3" t="inlineStr">
+        <is>
+          <t>Counsel answer with citation (REQUIREMENTS §9.2, FL Rule 64B8-10.002, R-3.8.2).</t>
+        </is>
+      </c>
+      <c r="H98" s="3" t="inlineStr">
+        <is>
+          <t>HC-3.7; HC-10.1; §9.2; ADR 0013</t>
+        </is>
+      </c>
+      <c r="I98" s="3" t="inlineStr">
+        <is>
+          <t>PR #107 session 2026-09-29</t>
+        </is>
+      </c>
+      <c r="J98" s="3" t="inlineStr">
+        <is>
+          <t>Before appeal attachments (A5)</t>
+        </is>
+      </c>
+      <c r="K98" s="3" t="inlineStr"/>
+      <c r="L98" s="3" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>OA-106</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>Approve PR #107 (ADR 0013 and HIPAA rules HC-3.5 to HC-3.9) in writing on the PR.</t>
+        </is>
+      </c>
+      <c r="F99" s="3" t="inlineStr">
+        <is>
+          <t>HC-13.2: an agent may not merge a change to HIPAA_COMPLIANCE.md without the owner's written approval in the PR.</t>
+        </is>
+      </c>
+      <c r="G99" s="3" t="inlineStr">
+        <is>
+          <t>A PR comment or approving review saying you approve.</t>
+        </is>
+      </c>
+      <c r="H99" s="3" t="inlineStr">
+        <is>
+          <t>HC-13.2; ADR 0013</t>
+        </is>
+      </c>
+      <c r="I99" s="3" t="inlineStr">
+        <is>
+          <t>PR #107 session 2026-09-29</t>
+        </is>
+      </c>
+      <c r="J99" s="3" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="K99" s="3" t="inlineStr"/>
+      <c r="L99" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L97"/>
+  <autoFilter ref="A1:L99"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Blocked,Done,Dropped"</formula1>

</xml_diff>

<commit_message>
docs(data-model): record owner approval of ADR 0013 and HC-3.5 to HC-3.9 [§9.2]
Owner approved the merge of PR #107 on 2026-09-29 (HC-13.2). ADR 0013 is
Accepted; OA-106 closed.

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TUv9KsDzYW8LQ1t8PjnRcr
</commit_message>
<xml_diff>
--- a/docs/owner/OWNER_ACTION_ITEMS.xlsx
+++ b/docs/owner/OWNER_ACTION_ITEMS.xlsx
@@ -6042,7 +6042,7 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
@@ -6086,7 +6086,11 @@
         </is>
       </c>
       <c r="K104" s="3" t="inlineStr"/>
-      <c r="L104" s="3" t="inlineStr"/>
+      <c r="L104" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L104"/>

</xml_diff>